<commit_message>
Resolve spinoff lot prices and fix CEDEAR data pipeline
Spinoff-only tickers (IRSA, ECOG) had avg_price=0.01 with no date or
FX rate, making P&L calculations impossible. Now the Balanz importer
preserves the spinoff date and MEP rate, and a new SpinoffPricer
service fetches the historical closing price from Data912.

- Balanz importer preserves date/mep for all-free lots
- SpinoffPricer resolves prices via Data912 historical API
- Handles abbreviated API keys (c vs close) and error hashes
- Strip .C suffix from BA.C when querying finance-query
- Fetch CEDEAR ratios from finance-query shortName field
- Document Data912 historical gotchas in finance-api skill
</commit_message>
<xml_diff>
--- a/spec/fixtures/balanz_sample.xlsx
+++ b/spec/fixtures/balanz_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -921,6 +921,61 @@
       </c>
       <c r="M9" t="n">
         <v>1100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IRSA INV.Y REPR. S.A.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>-13.97</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Pesos</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Split / CRES</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>IRSA</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Acciones</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1472.83</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1452.57</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>